<commit_message>
Update DRS question bank spreadsheet
Replace ASTquizApp/Data/QuestionBanks/DRS.xlsx with an updated Excel question bank (revised questions/answers and formatting). No code changes.

Co-authored-by: Copilot <223556219+Copilot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/ASTquizApp/Data/QuestionBanks/DRS.xlsx
+++ b/ASTquizApp/Data/QuestionBanks/DRS.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\programDo\vs\ASTquizApp\ASTquizApp\qBanks\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\programDo\vs\ASTquizApp\ASTquizApp\Data\QuestionBanks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF7B3F83-4D7D-437E-A7F8-E5B4FC1E855D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C7C8F27-1B08-4142-93FE-0B5B7D40C6C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -529,7 +529,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -1034,13 +1034,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O51"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.7109375" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.42578125" hidden="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="10" hidden="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="64.7109375" style="1" customWidth="1"/>
     <col min="9" max="9" width="21.140625" bestFit="1" customWidth="1"/>
@@ -1052,7 +1053,7 @@
     <col min="15" max="15" width="18.7109375" hidden="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="2" customFormat="1" ht="18.75">
+    <row r="1" spans="1:15" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1099,7 +1100,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:15" ht="60">
+    <row r="2" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>143</v>
       </c>
@@ -1146,7 +1147,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="3" spans="1:15" ht="60">
+    <row r="3" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>143</v>
       </c>
@@ -1193,7 +1194,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="4" spans="1:15" ht="60">
+    <row r="4" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>143</v>
       </c>
@@ -1240,7 +1241,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" spans="1:15" ht="60">
+    <row r="5" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>143</v>
       </c>
@@ -1283,7 +1284,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="6" spans="1:15" ht="60">
+    <row r="6" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>143</v>
       </c>
@@ -1330,7 +1331,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="7" spans="1:15" ht="60">
+    <row r="7" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>143</v>
       </c>
@@ -1377,7 +1378,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="8" spans="1:15" ht="60">
+    <row r="8" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>143</v>
       </c>
@@ -1424,7 +1425,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="9" spans="1:15" ht="60">
+    <row r="9" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>143</v>
       </c>
@@ -1471,7 +1472,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="10" spans="1:15" ht="60">
+    <row r="10" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>143</v>
       </c>
@@ -1518,7 +1519,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="11" spans="1:15" ht="60">
+    <row r="11" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>143</v>
       </c>
@@ -1565,7 +1566,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:15" ht="60">
+    <row r="12" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>143</v>
       </c>
@@ -1608,7 +1609,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:15" ht="60">
+    <row r="13" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>143</v>
       </c>
@@ -1655,7 +1656,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="14" spans="1:15" ht="60">
+    <row r="14" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>143</v>
       </c>
@@ -1698,7 +1699,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="15" spans="1:15" ht="60">
+    <row r="15" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>143</v>
       </c>
@@ -1745,7 +1746,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="16" spans="1:15" ht="60">
+    <row r="16" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>143</v>
       </c>
@@ -1788,7 +1789,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="17" spans="1:15" ht="60">
+    <row r="17" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>143</v>
       </c>
@@ -1835,7 +1836,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:15" ht="60">
+    <row r="18" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>143</v>
       </c>
@@ -1878,7 +1879,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="19" spans="1:15" ht="60">
+    <row r="19" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>143</v>
       </c>
@@ -1925,7 +1926,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="20" spans="1:15" ht="60">
+    <row r="20" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>143</v>
       </c>
@@ -1972,7 +1973,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:15" ht="60">
+    <row r="21" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A21" s="5" t="s">
         <v>143</v>
       </c>
@@ -2019,7 +2020,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="22" spans="1:15" ht="60">
+    <row r="22" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A22" s="5" t="s">
         <v>143</v>
       </c>
@@ -2066,7 +2067,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:15" ht="75">
+    <row r="23" spans="1:15" ht="75" x14ac:dyDescent="0.2">
       <c r="A23" s="5" t="s">
         <v>143</v>
       </c>
@@ -2113,7 +2114,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="24" spans="1:15" ht="60">
+    <row r="24" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A24" s="5" t="s">
         <v>143</v>
       </c>
@@ -2156,7 +2157,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:15" ht="60">
+    <row r="25" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A25" s="5" t="s">
         <v>143</v>
       </c>
@@ -2199,7 +2200,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:15" ht="60">
+    <row r="26" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A26" s="5" t="s">
         <v>143</v>
       </c>
@@ -2242,7 +2243,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="27" spans="1:15" ht="60">
+    <row r="27" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A27" s="5" t="s">
         <v>143</v>
       </c>
@@ -2285,7 +2286,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="28" spans="1:15" ht="60">
+    <row r="28" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A28" s="5" t="s">
         <v>143</v>
       </c>
@@ -2332,7 +2333,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="29" spans="1:15" ht="60">
+    <row r="29" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A29" s="5" t="s">
         <v>143</v>
       </c>
@@ -2375,7 +2376,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="30" spans="1:15" ht="60">
+    <row r="30" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A30" s="5" t="s">
         <v>143</v>
       </c>
@@ -2418,7 +2419,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="31" spans="1:15" ht="60">
+    <row r="31" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A31" s="5" t="s">
         <v>143</v>
       </c>
@@ -2461,7 +2462,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="60">
+    <row r="32" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A32" s="5" t="s">
         <v>143</v>
       </c>
@@ -2504,7 +2505,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="33" spans="1:15" ht="60">
+    <row r="33" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A33" s="5" t="s">
         <v>143</v>
       </c>
@@ -2547,7 +2548,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="34" spans="1:15" ht="60">
+    <row r="34" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A34" s="5" t="s">
         <v>143</v>
       </c>
@@ -2590,7 +2591,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="35" spans="1:15" ht="60">
+    <row r="35" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A35" s="5" t="s">
         <v>143</v>
       </c>
@@ -2637,7 +2638,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="36" spans="1:15" ht="60">
+    <row r="36" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A36" s="5" t="s">
         <v>143</v>
       </c>
@@ -2680,7 +2681,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="37" spans="1:15" ht="75">
+    <row r="37" spans="1:15" ht="75" x14ac:dyDescent="0.2">
       <c r="A37" s="5" t="s">
         <v>143</v>
       </c>
@@ -2727,7 +2728,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="38" spans="1:15" ht="60">
+    <row r="38" spans="1:15" ht="60" x14ac:dyDescent="0.2">
       <c r="A38" s="5" t="s">
         <v>143</v>
       </c>
@@ -2774,7 +2775,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="39" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="39" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A39" s="5" t="s">
         <v>143</v>
       </c>
@@ -2817,7 +2818,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="40" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="40" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A40" s="5" t="s">
         <v>143</v>
       </c>
@@ -2860,7 +2861,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="41" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="41" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A41" s="5" t="s">
         <v>143</v>
       </c>
@@ -2907,7 +2908,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="42" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="42" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A42" s="5" t="s">
         <v>143</v>
       </c>
@@ -2954,7 +2955,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="43" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="43" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A43" s="5" t="s">
         <v>143</v>
       </c>
@@ -3001,7 +3002,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="44" spans="1:15" s="18" customFormat="1" ht="105">
+    <row r="44" spans="1:15" s="18" customFormat="1" ht="105" x14ac:dyDescent="0.2">
       <c r="A44" s="5" t="s">
         <v>143</v>
       </c>
@@ -3048,7 +3049,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="45" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="45" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A45" s="5" t="s">
         <v>143</v>
       </c>
@@ -3091,7 +3092,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="46" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="46" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A46" s="5" t="s">
         <v>143</v>
       </c>
@@ -3134,7 +3135,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="47" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="47" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A47" s="5" t="s">
         <v>143</v>
       </c>
@@ -3181,7 +3182,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="48" spans="1:15" s="18" customFormat="1" ht="60">
+    <row r="48" spans="1:15" s="18" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A48" s="5" t="s">
         <v>143</v>
       </c>
@@ -3228,7 +3229,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="49" spans="1:15" s="20" customFormat="1" ht="60">
+    <row r="49" spans="1:15" s="20" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A49" s="21" t="s">
         <v>154</v>
       </c>
@@ -3275,7 +3276,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="50" spans="1:15" s="20" customFormat="1" ht="60">
+    <row r="50" spans="1:15" s="20" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A50" s="21" t="s">
         <v>154</v>
       </c>
@@ -3318,7 +3319,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:15" s="20" customFormat="1" ht="60">
+    <row r="51" spans="1:15" s="20" customFormat="1" ht="60" x14ac:dyDescent="0.2">
       <c r="A51" s="21" t="s">
         <v>154</v>
       </c>

</xml_diff>